<commit_message>
Add Flask endpoints (appp.py) — fix minti_app
</commit_message>
<xml_diff>
--- a/transactions.xlsx
+++ b/transactions.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,7 +492,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45967.19091825689</v>
+        <v>45967.19091825232</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -513,6 +513,32 @@
         </is>
       </c>
       <c r="F3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>45972.24832415008</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Clothing</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>200</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>New items</t>
+        </is>
+      </c>
+      <c r="F4" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>